<commit_message>
exp results strat eval
</commit_message>
<xml_diff>
--- a/results/reliability_eval/Llama-3-8B_P101_sample_15_tokens_0.1_temp_deductive_reasoning_scores_08-24-4.xlsx
+++ b/results/reliability_eval/Llama-3-8B_P101_sample_15_tokens_0.1_temp_deductive_reasoning_scores_08-24-4.xlsx
@@ -477,31 +477,31 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.5037788331071913</v>
+        <v>0.5585246088843211</v>
       </c>
       <c r="B2" t="n">
-        <v>0.3362739839583877</v>
+        <v>0.03291217553686192</v>
       </c>
       <c r="C2" t="n">
-        <v>0.5037788331071913</v>
+        <v>0.5585246088843211</v>
       </c>
       <c r="D2" t="n">
-        <v>0.3362739839583877</v>
+        <v>0.03291217553686192</v>
       </c>
       <c r="E2" t="n">
-        <v>0.5029149706015378</v>
+        <v>0.4417799094058087</v>
       </c>
       <c r="F2" t="n">
-        <v>0.3469024472300921</v>
+        <v>0.03097178683385579</v>
       </c>
       <c r="G2" t="n">
-        <v>0.9956580732700135</v>
+        <v>0.9988390240188801</v>
       </c>
       <c r="H2" t="n">
-        <v>0.98927875874372</v>
+        <v>0.9450617283950618</v>
       </c>
       <c r="I2" t="n">
-        <v>0.33</v>
+        <v>0.027</v>
       </c>
     </row>
   </sheetData>

</xml_diff>